<commit_message>
feat: verify rule CG0149 and add negative test cases
</commit_message>
<xml_diff>
--- a/rules/CORE-000088/negative/01/data/unit-test-coreid-CG0149-negative.xlsx
+++ b/rules/CORE-000088/negative/01/data/unit-test-coreid-CG0149-negative.xlsx
@@ -51,7 +51,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -62,6 +62,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFCC"/>
         <bgColor rgb="00FFFFCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -137,7 +143,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -163,6 +169,9 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -617,7 +626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -649,6 +658,118 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Error value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SETCD</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>DRUG_A_SMOKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>SETCD</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DRUG_B_SMOKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SETCD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>DRUG_A_NON_SMOKER</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>dm.xpt</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SETCD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>DRUG_B_NON_SMOKER</t>
         </is>
       </c>
     </row>
@@ -890,7 +1011,7 @@
           <t>Drug A</t>
         </is>
       </c>
-      <c r="J5" s="5" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>DRUG_A_SMOKER</t>
         </is>
@@ -932,7 +1053,7 @@
           <t>Drug B</t>
         </is>
       </c>
-      <c r="J6" s="5" t="inlineStr">
+      <c r="J6" s="10" t="inlineStr">
         <is>
           <t>DRUG_B_SMOKER</t>
         </is>
@@ -1053,7 +1174,7 @@
           <t>Drug A</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="10" t="inlineStr">
         <is>
           <t>DRUG_A_NON_SMOKER</t>
         </is>
@@ -1095,7 +1216,7 @@
           <t>Drug B</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="10" t="inlineStr">
         <is>
           <t>DRUG_B_NON_SMOKER</t>
         </is>

</xml_diff>